<commit_message>
fix: Correct item 89 SKU to 11-E-9851-02 on PO 65, support all 97 items in email body, and make dark banner 100% Outlook compatible with table bgcolor
</commit_message>
<xml_diff>
--- a/data/BD_POs_Partidas_Detalladas.xlsx
+++ b/data/BD_POs_Partidas_Detalladas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7412" uniqueCount="1390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7412" uniqueCount="1389">
   <si>
     <t>id_partida</t>
   </si>
@@ -1504,7 +1504,7 @@
     <t>11-E-9851-01</t>
   </si>
   <si>
-    <t>11-E-9851-02 - COMPARTIMIENTO AUXILIAR</t>
+    <t>11-E-9851-02</t>
   </si>
   <si>
     <t>11-E-9870-02</t>
@@ -4151,9 +4151,6 @@
   </si>
   <si>
     <t>SWB01941</t>
-  </si>
-  <si>
-    <t>11-E-9851-02</t>
   </si>
   <si>
     <t>ISSIV05319</t>
@@ -44342,7 +44339,7 @@
         <v>959</v>
       </c>
       <c r="M1048" t="s">
-        <v>1379</v>
+        <v>496</v>
       </c>
     </row>
     <row r="1049" spans="1:13">
@@ -44380,7 +44377,7 @@
         <v>959</v>
       </c>
       <c r="M1049" t="s">
-        <v>1380</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="1050" spans="1:13">
@@ -44418,7 +44415,7 @@
         <v>959</v>
       </c>
       <c r="M1050" t="s">
-        <v>1381</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="1051" spans="1:13">
@@ -44456,7 +44453,7 @@
         <v>959</v>
       </c>
       <c r="M1051" t="s">
-        <v>1382</v>
+        <v>1381</v>
       </c>
     </row>
     <row r="1052" spans="1:13">
@@ -44494,7 +44491,7 @@
         <v>959</v>
       </c>
       <c r="M1052" t="s">
-        <v>1383</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="1053" spans="1:13">
@@ -44532,7 +44529,7 @@
         <v>959</v>
       </c>
       <c r="M1053" t="s">
-        <v>1384</v>
+        <v>1383</v>
       </c>
     </row>
     <row r="1054" spans="1:13">
@@ -44570,7 +44567,7 @@
         <v>959</v>
       </c>
       <c r="M1054" t="s">
-        <v>1385</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="1055" spans="1:13">
@@ -44608,7 +44605,7 @@
         <v>959</v>
       </c>
       <c r="M1055" t="s">
-        <v>1386</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="1056" spans="1:13">
@@ -44646,7 +44643,7 @@
         <v>959</v>
       </c>
       <c r="M1056" t="s">
-        <v>1387</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="1057" spans="1:13">
@@ -44684,7 +44681,7 @@
         <v>959</v>
       </c>
       <c r="M1057" t="s">
-        <v>1388</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="1058" spans="1:13">
@@ -44722,7 +44719,7 @@
         <v>959</v>
       </c>
       <c r="M1058" t="s">
-        <v>1389</v>
+        <v>1388</v>
       </c>
     </row>
   </sheetData>

</xml_diff>